<commit_message>
chore(pubgen): refresh the bilingual sample set
The Dual Lang samples as the running app rewrites them: the publication note
(RTF) and the catalog workbook are re-saved, A03/A04 are gone and the English
variants of the chapter and review RTFs are in.
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
+++ b/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft\plan\pubgen\samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C000D459-01F6-4ED4-8D1C-55989C1A5B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{913B6D3C-E6D7-448F-9AD6-0BDBCB27D1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9600" yWindow="4770" windowWidth="28800" windowHeight="9285" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER" sheetId="7" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="74">
   <si>
     <t>Warungbambu</t>
   </si>
@@ -146,9 +146,6 @@
     <t>ISBN</t>
   </si>
   <si>
-    <t>BADAN PUSAT STATISTIK KABUPATEN KARAWANG</t>
-  </si>
-  <si>
     <t>image</t>
   </si>
   <si>
@@ -182,23 +179,14 @@
     <t>F:\Github\designcraft\plan\pubgen\samples\infografik_01.png</t>
   </si>
   <si>
-    <t>Tabel 01.01 Luas Daerah Menurut Desa/Kelurahan di Kecamatan  Karawang Timur, 2025</t>
-  </si>
-  <si>
     <t>Persentase terhadap Luas Kecamatan</t>
   </si>
   <si>
-    <t>Desa/Village</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Kelurahan/Subdistrict</t>
-  </si>
-  <si>
     <t>/ Percentage to District Area</t>
   </si>
   <si>
     <r>
-      <t>(km2</t>
+      <t xml:space="preserve">Luas / </t>
     </r>
     <r>
       <rPr>
@@ -209,13 +197,243 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>/sq.km</t>
-    </r>
-    <r>
-      <rPr>
+      <t>Total Area</t>
+    </r>
+  </si>
+  <si>
+    <t>Desa/Kelurahan / Village/Subdistric</t>
+  </si>
+  <si>
+    <t>diivider</t>
+  </si>
+  <si>
+    <t>dividers/special_infographic_divider</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01.rtf</t>
+  </si>
+  <si>
+    <t>KECAMATAN KARAWANG TIMUR</t>
+  </si>
+  <si>
+    <t>DALAM ANGKA</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01.rtf</t>
+  </si>
+  <si>
+    <t>image2</t>
+  </si>
+  <si>
+    <t>image1</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict1.jpg</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
+  </si>
+  <si>
+    <t>file_en</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Kata Pengantar / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
         <sz val="10"/>
         <color rgb="FF000000"/>
         <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Preface</t>
+    </r>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_en.rtf</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BAB / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Chapter </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 01 GEOGRAFI / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>GEOGRAPHY</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Bab / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Chapter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 01  Geografi / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Geography</t>
+    </r>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01_en.rtf</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Tabel 01.01 Luas Daerah Menurut Desa/Kelurahan di Kecamatan  Karawang Timur / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Land Area by Village/Sub-district in East Karawang District</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 2025</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Desa / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Village</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> Kelurahan / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Subdistrict</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Kec. / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dist.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Karawang Timur</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>(km2 /</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> sq.km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>)</t>
@@ -223,7 +441,9 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Luas / </t>
+      <t xml:space="preserve">BADAN PUSAT STATISTIK
+KABUPATEN KARAWANG
+</t>
     </r>
     <r>
       <rPr>
@@ -234,60 +454,15 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Total Area</t>
-    </r>
-  </si>
-  <si>
-    <t>Kec. Karawang Timur</t>
-  </si>
-  <si>
-    <t>Desa/Kelurahan / Village/Subdistric</t>
-  </si>
-  <si>
-    <t>BAB 01 GEOGRAFI</t>
-  </si>
-  <si>
-    <t>diivider</t>
-  </si>
-  <si>
-    <t>dividers/special_infographic_divider</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01.rtf</t>
-  </si>
-  <si>
-    <t>KECAMATAN KARAWANG TIMUR</t>
-  </si>
-  <si>
-    <t>DALAM ANGKA</t>
-  </si>
-  <si>
-    <t>Bab 01  Geografi</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01.rtf</t>
-  </si>
-  <si>
-    <t>image2</t>
-  </si>
-  <si>
-    <t>image1</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict1.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
-  </si>
-  <si>
-    <t>Kata Pengantar</t>
+      <t>Central Statistics Agency Of Karawang Regency</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -310,6 +485,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -694,7 +876,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -702,7 +884,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -737,12 +919,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
-        <v>37</v>
+      <c r="B8" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -750,7 +932,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -758,7 +940,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -766,7 +948,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -879,7 +1061,7 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -900,7 +1082,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -918,7 +1100,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -936,7 +1118,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -946,39 +1128,47 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7036A343-3A5A-488B-8DC0-22E63F44947D}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
-        <v>70</v>
+      <c r="B1" s="1" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>65</v>
+      <c r="B2" s="1" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" t="s">
-        <v>68</v>
+      <c r="A3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -996,23 +1186,23 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1022,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6A079BF-B32C-4911-B14D-3B9A331ACB0B}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5703125" style="11" bestFit="1" customWidth="1"/>
@@ -1034,7 +1224,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1042,15 +1232,23 @@
         <v>9</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>60</v>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1070,19 +1268,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -1090,17 +1288,17 @@
     <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="12"/>
       <c r="B3" s="9" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>51</v>
+      <c r="A4" s="8" t="s">
+        <v>69</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -1150,8 +1348,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>52</v>
+      <c r="A9" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -1202,7 +1400,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="8" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="B14" s="7">
         <f>SUM(B4:B13)</f>

</xml_diff>

<commit_message>
pubgen: keep Excel multiline table cells as line breaks
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
+++ b/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
@@ -5,20 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft-modular\plan\pubgen\samples\DUAL_LANG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\pubgen-bilingual\plan\pubgen\samples\DUAL_LANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B30813D6-2CFE-4E1C-A417-72D184067894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758229E6-E13F-499D-A117-F3FC19B0F908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6690" yWindow="6435" windowWidth="28800" windowHeight="9285" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER" sheetId="7" r:id="rId1"/>
     <sheet name="A02" sheetId="6" r:id="rId2"/>
     <sheet name="G00" sheetId="10" r:id="rId3"/>
-    <sheet name="G01" sheetId="11" r:id="rId4"/>
-    <sheet name="G02" sheetId="12" r:id="rId5"/>
-    <sheet name="B01" sheetId="15" r:id="rId6"/>
+    <sheet name="B01" sheetId="15" r:id="rId4"/>
+    <sheet name="G01" sheetId="11" r:id="rId5"/>
+    <sheet name="G02" sheetId="12" r:id="rId6"/>
     <sheet name="DIV" sheetId="9" r:id="rId7"/>
     <sheet name="R01" sheetId="14" r:id="rId8"/>
     <sheet name="01_01" sheetId="13" r:id="rId9"/>
@@ -29,11 +29,22 @@
     <definedName name="_Toc202275225" localSheetId="8">'01_01'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="75">
   <si>
     <t>Warungbambu</t>
   </si>
@@ -177,28 +188,6 @@
   </si>
   <si>
     <t>F:\Github\designcraft\plan\pubgen\samples\infografik_01.png</t>
-  </si>
-  <si>
-    <t>Persentase terhadap Luas Kecamatan</t>
-  </si>
-  <si>
-    <t>/ Percentage to District Area</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Luas / </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Total Area</t>
-    </r>
   </si>
   <si>
     <t>Desa/Kelurahan / Village/Subdistric</t>
@@ -365,32 +354,6 @@
   </si>
   <si>
     <r>
-      <t>(km2 /</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> sq.km</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">BADAN PUSAT STATISTIK
 KABUPATEN KARAWANG
 </t>
@@ -421,6 +384,12 @@
   </si>
   <si>
     <t>Chapter 01 Geography</t>
+  </si>
+  <si>
+    <t>Luas / Total Area (km2 / sq.km)</t>
+  </si>
+  <si>
+    <t>Persentase terhadap Luas Kecamatan / Percentage to District Area</t>
   </si>
 </sst>
 </file>
@@ -483,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
@@ -502,12 +471,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -843,7 +806,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -851,7 +814,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -891,7 +854,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -1058,6 +1021,64 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7036A343-3A5A-488B-8DC0-22E63F44947D}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F26592-D980-4158-B6B2-66708CA1DAA0}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -1075,7 +1096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CF380A0-4220-41D5-9D63-0F4EABAFF4D6}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -1086,64 +1107,6 @@
       </c>
       <c r="B1" t="s">
         <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7036A343-3A5A-488B-8DC0-22E63F44947D}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>74</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1161,7 +1124,7 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1190,48 +1153,48 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7" style="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="11"/>
+    <col min="1" max="1" width="7" style="9" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="11" t="s">
-        <v>75</v>
+      <c r="B1" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>76</v>
+      <c r="A2" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>54</v>
+      <c r="B3" s="9" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>65</v>
-      </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>53</v>
+      <c r="A5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1242,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E203F7C2-8B4E-4514-90A6-3C366D18C374}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.140625" customWidth="1"/>
@@ -1252,153 +1215,137 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
-        <v>51</v>
+      <c r="A2" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="1:5" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="14"/>
-      <c r="B3" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
+      <c r="A4" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7">
+        <v>1.65</v>
+      </c>
+      <c r="C4" s="7">
+        <v>21.32</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="7">
-        <v>1.65</v>
+        <v>2.44</v>
       </c>
       <c r="C5" s="7">
-        <v>21.32</v>
+        <v>8.84</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" s="7">
-        <v>2.44</v>
+        <v>2.76</v>
       </c>
       <c r="C6" s="7">
-        <v>8.84</v>
+        <v>7.17</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B7" s="7">
-        <v>2.76</v>
+        <v>4.38</v>
       </c>
       <c r="C7" s="7">
-        <v>7.17</v>
+        <v>13.48</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="7">
-        <v>4.38</v>
-      </c>
-      <c r="C8" s="7">
-        <v>13.48</v>
-      </c>
+      <c r="A8" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
+      <c r="A9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7">
+        <v>4.32</v>
+      </c>
+      <c r="C9" s="7">
+        <v>17.27</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="7">
-        <v>4.32</v>
+        <v>3.2</v>
       </c>
       <c r="C10" s="7">
-        <v>17.27</v>
+        <v>7.91</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" s="7">
-        <v>3.2</v>
+        <v>4.0199999999999996</v>
       </c>
       <c r="C11" s="7">
-        <v>7.91</v>
+        <v>11.87</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12" s="7">
-        <v>4.0199999999999996</v>
+        <v>7</v>
       </c>
       <c r="C12" s="7">
-        <v>11.87</v>
+        <v>12.14</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>7</v>
+      <c r="A13" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="B13" s="7">
-        <v>7</v>
+        <v>29.77</v>
       </c>
       <c r="C13" s="7">
-        <v>12.14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="B14" s="7">
-        <f>SUM(B4:B13)</f>
-        <v>29.77</v>
-      </c>
-      <c r="C14" s="7">
-        <f>SUM(C4:C13)</f>
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:A3"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
update file sample for Dual Lang
</commit_message>
<xml_diff>
--- a/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
+++ b/plan/pubgen/samples/DUAL_LANG/BAB_01_2025.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Github\pubgen-bilingual\plan\pubgen\samples\DUAL_LANG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{758229E6-E13F-499D-A117-F3FC19B0F908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2877AB43-CF21-45B2-B403-407C0EDC2A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COVER" sheetId="7" r:id="rId1"/>
@@ -29,22 +29,11 @@
     <definedName name="_Toc202275225" localSheetId="8">'01_01'!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
   <si>
     <t>Warungbambu</t>
   </si>
@@ -166,30 +155,6 @@
     <t>002</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G00.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G01.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\G02.rtf</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\city_skyline.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\city_landscape.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\images\bps_logo.png</t>
-  </si>
-  <si>
-    <t>F:\Github\designcraft\plan\pubgen\samples\A02.rtf</t>
-  </si>
-  <si>
-    <t>F:\Github\designcraft\plan\pubgen\samples\infografik_01.png</t>
-  </si>
-  <si>
     <t>Desa/Kelurahan / Village/Subdistric</t>
   </si>
   <si>
@@ -199,39 +164,183 @@
     <t>dividers/special_infographic_divider</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01.rtf</t>
-  </si>
-  <si>
-    <t>KECAMATAN KARAWANG TIMUR</t>
-  </si>
-  <si>
-    <t>DALAM ANGKA</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01.rtf</t>
-  </si>
-  <si>
     <t>image2</t>
   </si>
   <si>
     <t>image1</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict1.jpg</t>
-  </si>
-  <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_pict2.png</t>
-  </si>
-  <si>
     <t>file_en</t>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\B01_en.rtf</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">BAB / </t>
-    </r>
+    <r>
+      <t xml:space="preserve">Tabel 01.01 Luas Daerah Menurut Desa/Kelurahan di Kecamatan  Karawang Timur / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Land Area by Village/Sub-district in East Karawang District</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 2025</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Desa / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Village</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve"> Kelurahan / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Subdistrict</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Kec. / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dist.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Karawang Timur</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">BADAN PUSAT STATISTIK
+KABUPATEN KARAWANG
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Central Statistics Agency Of Karawang Regency</t>
+    </r>
+  </si>
+  <si>
+    <t>Kata Pengantar</t>
+  </si>
+  <si>
+    <t>Preface</t>
+  </si>
+  <si>
+    <t>title_en</t>
+  </si>
+  <si>
+    <t>Bab 01 Geografi</t>
+  </si>
+  <si>
+    <t>Chapter 01 Geography</t>
+  </si>
+  <si>
+    <t>Luas / Total Area (km2 / sq.km)</t>
+  </si>
+  <si>
+    <t>Persentase terhadap Luas Kecamatan / Percentage to District Area</t>
+  </si>
+  <si>
+    <t>KECAMATAN KARAWANG TIMUR DALAM ANGKA</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\R01.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\R01_en.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\infografik_01.png</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\G02.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\G01.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\B01.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\B01_en.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\B01_pict1.jpg</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\B01_pict2.png</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\G00.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\A02.rtf</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\images\city_skyline.jpg</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\images\city_landscape.jpg</t>
+  </si>
+  <si>
+    <t>F:\GitHub\designcraft\plan\pubgen\samples\DUAL_LANG\images\bps_logo.png</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <i/>
@@ -251,7 +360,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> 01 GEOGRAFI / </t>
+      <t xml:space="preserve">01 </t>
     </r>
     <r>
       <rPr>
@@ -266,130 +375,7 @@
     </r>
   </si>
   <si>
-    <t>F:\GitHub\designcraft\plan\pubgen\samples\R01_en.rtf</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Tabel 01.01 Luas Daerah Menurut Desa/Kelurahan di Kecamatan  Karawang Timur / </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Land Area by Village/Sub-district in East Karawang District</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 2025</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Desa / </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Village</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> Kelurahan / </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Subdistrict</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Kec. / </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Dist.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Karawang Timur</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">BADAN PUSAT STATISTIK
-KABUPATEN KARAWANG
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Central Statistics Agency Of Karawang Regency</t>
-    </r>
-  </si>
-  <si>
-    <t>Kata Pengantar</t>
-  </si>
-  <si>
-    <t>Preface</t>
-  </si>
-  <si>
-    <t>title_en</t>
-  </si>
-  <si>
-    <t>Bab 01 Geografi</t>
-  </si>
-  <si>
-    <t>Chapter 01 Geography</t>
-  </si>
-  <si>
-    <t>Luas / Total Area (km2 / sq.km)</t>
-  </si>
-  <si>
-    <t>Persentase terhadap Luas Kecamatan / Percentage to District Area</t>
+    <t>BAB 01 GEOGRAFI</t>
   </si>
 </sst>
 </file>
@@ -806,16 +792,13 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -854,7 +837,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>67</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -862,7 +845,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -870,7 +853,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -878,7 +861,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -991,7 +974,7 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1012,7 +995,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1030,15 +1013,15 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>69</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1046,31 +1029,31 @@
         <v>9</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1088,7 +1071,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1106,7 +1089,7 @@
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AD23214-2BBD-426B-B52A-7BD7906A7070}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -1124,22 +1107,30 @@
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>47</v>
+        <v>53</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1162,15 +1153,15 @@
         <v>8</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>71</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1178,23 +1169,23 @@
         <v>9</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1215,26 +1206,26 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>73</v>
+        <v>56</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -1285,7 +1276,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -1336,7 +1327,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="8" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="B13" s="7">
         <v>29.77</v>

</xml_diff>